<commit_message>
add bet to print
</commit_message>
<xml_diff>
--- a/winner_final/data/wnba.xlsx
+++ b/winner_final/data/wnba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dkdk1\PycharmProjects\PythonProjectNew\winner_final\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C79135-0321-457D-AEFA-0B6068CA6BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC219CDD-FC91-4949-B2C9-6EA7126441F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1236" yWindow="1008" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Atlanta Dream</t>
   </si>
@@ -124,6 +124,12 @@
   </si>
   <si>
     <t>אינדיאנה פיבר</t>
+  </si>
+  <si>
+    <t>פורטלנד פייר</t>
+  </si>
+  <si>
+    <t>Portland Fire</t>
   </si>
 </sst>
 </file>
@@ -474,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.8984375" customWidth="1"/>
@@ -690,6 +696,20 @@
       <c r="C16" t="s">
         <v>5</v>
       </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="3">
+        <v>22</v>
+      </c>
+      <c r="C17" t="s">
+        <v>33</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>